<commit_message>
mise a jour requete produits
</commit_message>
<xml_diff>
--- a/produits.xlsx
+++ b/produits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOEL\Documents\python projects\intermediaire\Gestock App2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF0B8D65-657E-4C7D-88C1-B6F0D6F28CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{630EBD7F-9203-42C4-A879-0D117F120BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C3931086-43D5-4A52-A6E8-962A3A8F80E3}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="88">
   <si>
     <t>nom_produit</t>
   </si>
@@ -241,13 +241,61 @@
   </si>
   <si>
     <t>Description pour Film DI-HL 35X43</t>
+  </si>
+  <si>
+    <t>marque</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>origine</t>
+  </si>
+  <si>
+    <t>POLOGNE</t>
+  </si>
+  <si>
+    <t>JAPON</t>
+  </si>
+  <si>
+    <t>ARABIE S.</t>
+  </si>
+  <si>
+    <t>FRANCE</t>
+  </si>
+  <si>
+    <t>INDIA</t>
+  </si>
+  <si>
+    <t>CHINA</t>
+  </si>
+  <si>
+    <t>ITALIE</t>
+  </si>
+  <si>
+    <t>DUBAI</t>
+  </si>
+  <si>
+    <t>EZy-RAD Pro</t>
+  </si>
+  <si>
+    <t>OPTOPOL</t>
+  </si>
+  <si>
+    <t>SHIMADZU</t>
+  </si>
+  <si>
+    <t>FUJIFILM</t>
+  </si>
+  <si>
+    <t>VATECH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -261,13 +309,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -282,8 +343,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -598,299 +661,469 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D654166F-2DB8-4A57-BEC6-3E7FAE1DC896}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C3" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C4" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E5" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C6" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E7" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E8" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
       <c r="B9" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E10" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
       <c r="B11" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E11" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
       <c r="B12" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E12" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E13" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="B14" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E14" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>
       <c r="B15" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E15" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>16</v>
       </c>
       <c r="B16" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E16" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E17" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>18</v>
       </c>
       <c r="B18" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E18" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>19</v>
       </c>
       <c r="B19" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C19" t="s">
+        <v>86</v>
+      </c>
+      <c r="D19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>20</v>
       </c>
       <c r="B20" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C20" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>21</v>
       </c>
       <c r="B21" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E21" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>22</v>
       </c>
       <c r="B22" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E22" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>23</v>
       </c>
       <c r="B23" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E23" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>24</v>
       </c>
       <c r="B24" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E24" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>25</v>
       </c>
       <c r="B25" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E25" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>26</v>
       </c>
       <c r="B26" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E26" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>27</v>
       </c>
       <c r="B27" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E27" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>28</v>
       </c>
       <c r="B28" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E28" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>29</v>
       </c>
       <c r="B29" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E29" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>30</v>
       </c>
       <c r="B30" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E30" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>31</v>
       </c>
       <c r="B31" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C31" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>32</v>
       </c>
       <c r="B32" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C32" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" t="s">
+        <v>32</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>33</v>
       </c>
       <c r="B33" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E33" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>34</v>
       </c>
       <c r="B34" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E34" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>35</v>
       </c>
       <c r="B35" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="E35" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>36</v>
       </c>
       <c r="B36" t="s">
         <v>71</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mise a jour requete produits 1
</commit_message>
<xml_diff>
--- a/produits.xlsx
+++ b/produits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JOEL\Documents\python projects\intermediaire\Gestock App2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{630EBD7F-9203-42C4-A879-0D117F120BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A8D5A82-7A5D-4DEB-A589-11AD0326A670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C3931086-43D5-4A52-A6E8-962A3A8F80E3}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="92">
   <si>
     <t>nom_produit</t>
   </si>
@@ -289,6 +289,18 @@
   </si>
   <si>
     <t>VATECH</t>
+  </si>
+  <si>
+    <t>UNIJULE</t>
+  </si>
+  <si>
+    <t>SHANDONG</t>
+  </si>
+  <si>
+    <t>METALTRONICA</t>
+  </si>
+  <si>
+    <t>AOHUA</t>
   </si>
 </sst>
 </file>
@@ -666,6 +678,7 @@
   <cols>
     <col min="1" max="1" width="29.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.36328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.08984375" bestFit="1" customWidth="1"/>
   </cols>
@@ -745,6 +758,9 @@
       <c r="B5" t="s">
         <v>40</v>
       </c>
+      <c r="C5" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E5" s="1" t="s">
         <v>77</v>
       </c>
@@ -773,6 +789,9 @@
       <c r="B7" t="s">
         <v>42</v>
       </c>
+      <c r="C7" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="E7" s="1" t="s">
         <v>79</v>
       </c>
@@ -784,6 +803,9 @@
       <c r="B8" t="s">
         <v>43</v>
       </c>
+      <c r="C8" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="E8" s="1" t="s">
         <v>79</v>
       </c>
@@ -812,6 +834,9 @@
       <c r="B10" t="s">
         <v>45</v>
       </c>
+      <c r="C10" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E10" s="1" t="s">
         <v>80</v>
       </c>
@@ -823,6 +848,9 @@
       <c r="B11" t="s">
         <v>46</v>
       </c>
+      <c r="C11" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E11" s="1" t="s">
         <v>80</v>
       </c>
@@ -834,6 +862,9 @@
       <c r="B12" t="s">
         <v>47</v>
       </c>
+      <c r="C12" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E12" s="1" t="s">
         <v>80</v>
       </c>
@@ -845,6 +876,9 @@
       <c r="B13" t="s">
         <v>48</v>
       </c>
+      <c r="C13" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E13" s="1" t="s">
         <v>80</v>
       </c>
@@ -856,6 +890,9 @@
       <c r="B14" t="s">
         <v>49</v>
       </c>
+      <c r="C14" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E14" s="1" t="s">
         <v>80</v>
       </c>
@@ -867,6 +904,9 @@
       <c r="B15" t="s">
         <v>50</v>
       </c>
+      <c r="C15" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E15" s="1" t="s">
         <v>80</v>
       </c>
@@ -878,6 +918,9 @@
       <c r="B16" t="s">
         <v>51</v>
       </c>
+      <c r="C16" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E16" s="1" t="s">
         <v>80</v>
       </c>
@@ -889,6 +932,9 @@
       <c r="B17" t="s">
         <v>52</v>
       </c>
+      <c r="C17" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E17" s="1" t="s">
         <v>80</v>
       </c>
@@ -900,6 +946,9 @@
       <c r="B18" t="s">
         <v>53</v>
       </c>
+      <c r="C18" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="E18" s="1" t="s">
         <v>80</v>
       </c>
@@ -911,7 +960,7 @@
       <c r="B19" t="s">
         <v>54</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D19" t="s">
@@ -928,7 +977,7 @@
       <c r="B20" t="s">
         <v>55</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D20" t="s">
@@ -945,6 +994,9 @@
       <c r="B21" t="s">
         <v>56</v>
       </c>
+      <c r="C21" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E21" s="1" t="s">
         <v>77</v>
       </c>
@@ -956,6 +1008,9 @@
       <c r="B22" t="s">
         <v>57</v>
       </c>
+      <c r="C22" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E22" s="1" t="s">
         <v>77</v>
       </c>
@@ -967,6 +1022,9 @@
       <c r="B23" t="s">
         <v>58</v>
       </c>
+      <c r="C23" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E23" s="1" t="s">
         <v>77</v>
       </c>
@@ -978,6 +1036,9 @@
       <c r="B24" t="s">
         <v>59</v>
       </c>
+      <c r="C24" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E24" s="1" t="s">
         <v>77</v>
       </c>
@@ -989,6 +1050,9 @@
       <c r="B25" t="s">
         <v>60</v>
       </c>
+      <c r="C25" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E25" s="1" t="s">
         <v>77</v>
       </c>
@@ -1000,6 +1064,9 @@
       <c r="B26" t="s">
         <v>61</v>
       </c>
+      <c r="C26" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E26" s="1" t="s">
         <v>77</v>
       </c>
@@ -1011,6 +1078,9 @@
       <c r="B27" t="s">
         <v>62</v>
       </c>
+      <c r="C27" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E27" s="1" t="s">
         <v>77</v>
       </c>
@@ -1022,6 +1092,9 @@
       <c r="B28" t="s">
         <v>63</v>
       </c>
+      <c r="C28" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E28" s="1" t="s">
         <v>77</v>
       </c>
@@ -1033,6 +1106,9 @@
       <c r="B29" t="s">
         <v>64</v>
       </c>
+      <c r="C29" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E29" s="1" t="s">
         <v>77</v>
       </c>
@@ -1044,6 +1120,9 @@
       <c r="B30" t="s">
         <v>65</v>
       </c>
+      <c r="C30" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E30" s="1" t="s">
         <v>77</v>
       </c>
@@ -1055,7 +1134,7 @@
       <c r="B31" t="s">
         <v>66</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D31" t="s">
@@ -1072,7 +1151,7 @@
       <c r="B32" t="s">
         <v>67</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D32" t="s">
@@ -1089,6 +1168,9 @@
       <c r="B33" t="s">
         <v>68</v>
       </c>
+      <c r="C33" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="E33" s="1" t="s">
         <v>81</v>
       </c>
@@ -1100,6 +1182,9 @@
       <c r="B34" t="s">
         <v>69</v>
       </c>
+      <c r="C34" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="E34" s="1" t="s">
         <v>80</v>
       </c>
@@ -1111,6 +1196,9 @@
       <c r="B35" t="s">
         <v>70</v>
       </c>
+      <c r="C35" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="E35" s="1" t="s">
         <v>82</v>
       </c>
@@ -1121,6 +1209,9 @@
       </c>
       <c r="B36" t="s">
         <v>71</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>82</v>

</xml_diff>